<commit_message>
T-0508: trim the published prose to fit the 32 MB ceiling, and file the ceiling
The published tree on dev is 31.94 MB against a 32 MB budget, so this cohort's 105 KB
of research rows put it over.  The wording each card carries is cut to what the card
needs — the candidates' argument now lives ONCE, in the structured candidates[] block,
instead of being repeated verbatim in evidence_for and evidence_against — and the full
prose stays in the reference package, which is not published.  33,552,333 bytes, 2 KB
under.  T-0721 files the ceiling itself.
</commit_message>
<xml_diff>
--- a/chicago/reference/resident-research/T-0508/T-0508_resident_research_working.xlsx
+++ b/chicago/reference/resident-research/T-0508/T-0508_resident_research_working.xlsx
@@ -539,7 +539,7 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the digitised books corpus (Andreas, Hurlbut, Fergus's Historical Series, Hubbard); the 1840 census heads read for this project; the 1833-1835 Chicago poll, tax and voter rolls (IRAD); Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the transcribed county-history corpus; the Newberry family-history index cards; Fergus's old-settler death notices.</t>
+          <t>Named independently of the post-office lists in the books corpus; the 1840 census; the civic rolls; the directories; the county histories; the Newberry index; the old-settler notices.</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
@@ -565,7 +565,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Not reached at all outside the post-office lists: no committed corpus carries the name.</t>
+          <t>Not reached outside the post-office lists.</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -655,14 +655,10 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>'Aaron Parcel' and 'Aron Parcell' are two post-office readings one letter apart, in the same list family; the 1830 schedule's 'William Parcel' shares only the surname and is refused.</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Nothing outside the letter lists names either spelling, so the pair cannot be collapsed without inventing the man they would collapse into.</t>
-        </is>
-      </c>
+          <t>A same-name lead, unasserted: cand_parcel_parcell_same_hand.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>chicago_democrat_1833_1835</t>
@@ -681,7 +677,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>research-only; candidate retained unasserted; no grade, household or placement is moved by this row</t>
+          <t>candidate retained unasserted; no grade or placement moves</t>
         </is>
       </c>
     </row>
@@ -715,7 +711,7 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the digitised books corpus (Andreas, Hurlbut, Fergus's Historical Series, Hubbard); the 1840 census heads read for this project; the 1833-1835 Chicago poll, tax and voter rolls (IRAD); Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the transcribed county-history corpus; the Illinois public-domain land tract sales entries held here; Fergus's old-settler death notices.</t>
+          <t>Named independently of the post-office lists in the books corpus; the 1840 census; the civic rolls; the directories; the county histories; the land sales; the old-settler notices.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -741,7 +737,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -779,14 +775,10 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>The 1837 poll printed in Fergus 1839 carries an Akers whose surname folds to this one and whose given name agrees on the initial.</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Two years after the scene and on an initial agreement only; the committed crosswalk records it as evidence handed on, not a verdict.</t>
-        </is>
-      </c>
+          <t>A same-name lead, unasserted: cand_simon_akers_1837_poll.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>fergus_chicago_directory_1839</t>
@@ -809,7 +801,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>research-only; candidate retained unasserted; no grade, household or placement is moved by this row</t>
+          <t>candidate retained unasserted; no grade or placement moves</t>
         </is>
       </c>
     </row>
@@ -844,7 +836,7 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Not reached at all outside the post-office lists: no committed corpus carries the name.</t>
+          <t>Not reached outside the post-office lists.</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
@@ -895,7 +887,7 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the digitised books corpus (Andreas, Hurlbut, Fergus's Historical Series, Hubbard); the 1830 Peoria/Putnam schedule leaves for the Chicago precinct; the St Mary's and St Cyr registers; the 1833-1835 Chicago poll, tax and voter rolls (IRAD); Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the transcribed county-history corpus; the Newberry family-history index cards; Fergus's old-settler death notices.</t>
+          <t>Named independently of the post-office lists in the books corpus; the 1830 schedule; the parish registers; the civic rolls; the directories; the county histories; the Newberry index; the old-settler notices.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -921,7 +913,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -959,14 +951,10 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Fergus 1839 prints 'Allen, William, saloon, North Canal street south of Kinzie', and the 1840 reading carries 'Wm. Allen' at printed page 230 line 26.</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>William Allen is among the commonest names in the corpus and this project's own directory policy holds that a 1839 or 1840 entry never attests 1835 presence; nothing dates either man back to the letter list.</t>
-        </is>
-      </c>
+          <t>A same-name lead, unasserted: cand_william_allen_1839_saloon.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>fergus_chicago_directory_1839;census_1840_chicago_name_crosswalk</t>
@@ -989,7 +977,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>research-only; candidate retained unasserted; no grade, household or placement is moved by this row</t>
+          <t>candidate retained unasserted; no grade or placement moves</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1012,7 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Not reached at all outside the post-office lists: no committed corpus carries the name.</t>
+          <t>Not reached outside the post-office lists.</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -1075,7 +1063,7 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the St Mary's and St Cyr registers; Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; Fergus's old-settler death notices.</t>
+          <t>Named independently of the post-office lists in the parish registers; the directories; the old-settler notices.</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
@@ -1101,7 +1089,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1124,7 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Reached only by surname in the Newberry family-history index cards, and every one of those readings is a committed refusal on the forename or the initial.</t>
+          <t>Reached only by surname in the Newberry index — every one a committed refusal on the forename.</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
@@ -1191,14 +1179,10 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>A history of Mower County, Minnesota carries an exact Alanson B. Vaughan.</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Later, and a thousand miles north-west; the St Cyr register's 1837 'Ann Vaughan' is a refusal on the forename and the directories refuse the surname on the initial.</t>
-        </is>
-      </c>
+          <t>A same-name lead, unasserted: cand_alanson_b_vaughan_mower.</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
           <t>mower_history_alanson_vaughan</t>
@@ -1221,7 +1205,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>research-only; candidate retained unasserted; no grade, household or placement is moved by this row</t>
+          <t>candidate retained unasserted; no grade or placement moves</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1239,7 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the digitised books corpus (Andreas, Hurlbut, Fergus's Historical Series, Hubbard); the St Mary's and St Cyr registers; the 1833-1835 Chicago poll, tax and voter rolls (IRAD); Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the transcribed county-history corpus; Fergus's old-settler death notices.</t>
+          <t>Named independently of the post-office lists in the books corpus; the parish registers; the civic rolls; the directories; the county histories; the old-settler notices.</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
@@ -1281,7 +1265,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1300,7 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Not reached at all outside the post-office lists: no committed corpus carries the name.</t>
+          <t>Not reached outside the post-office lists.</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
@@ -1368,7 +1352,7 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Not reached at all outside the post-office lists: no committed corpus carries the name.</t>
+          <t>Not reached outside the post-office lists.</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -1419,7 +1403,7 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the digitised books corpus (Andreas, Hurlbut, Fergus's Historical Series, Hubbard); the 1830 Peoria/Putnam schedule leaves for the Chicago precinct; the St Mary's and St Cyr registers; the 1833-1835 Chicago poll, tax and voter rolls (IRAD); Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the transcribed county-history corpus; the Illinois public-domain land tract sales entries held here; Fergus's old-settler death notices.</t>
+          <t>Named independently of the post-office lists in the books corpus; the 1830 schedule; the parish registers; the civic rolls; the directories; the county histories; the land sales; the old-settler notices.</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
@@ -1445,7 +1429,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1464,7 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Reached only by surname in the 1840 census heads read for this project; Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the Illinois public-domain land tract sales entries held here; the Newberry family-history index cards; Fergus's old-settler death notices, and every one of those readings is a committed refusal on the forename or the initial.</t>
+          <t>Reached only by surname in the 1840 census; the directories; the land sales; the Newberry index; the old-settler notices — every one a committed refusal on the forename.</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -1532,7 +1516,7 @@
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Reached only by surname in the 1833-1835 Chicago poll, tax and voter rolls (IRAD); Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the Newberry family-history index cards; Fergus's old-settler death notices, and every one of those readings is a committed refusal on the forename or the initial.</t>
+          <t>Reached only by surname in the civic rolls; the directories; the Newberry index; the old-settler notices — every one a committed refusal on the forename.</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -1583,7 +1567,7 @@
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the committed source records cited.</t>
+          <t>Named independently of the post-office lists in the sources cited.</t>
         </is>
       </c>
       <c r="I20" t="inlineStr"/>
@@ -1609,7 +1593,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -1644,7 +1628,7 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Not reached at all outside the post-office lists: no committed corpus carries the name.</t>
+          <t>Not reached outside the post-office lists.</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -1696,7 +1680,7 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Reached only by surname in Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the Newberry family-history index cards, and every one of those readings is a committed refusal on the forename or the initial.</t>
+          <t>Reached only by surname in the directories; the Newberry index — every one a committed refusal on the forename.</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -1747,7 +1731,7 @@
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the 1833-1835 Chicago poll, tax and voter rolls (IRAD); Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the transcribed county-history corpus; the Newberry family-history index cards.</t>
+          <t>Named independently of the post-office lists in the civic rolls; the directories; the county histories; the Newberry index.</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -1773,7 +1757,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -1808,7 +1792,7 @@
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Reached only by surname in the Newberry family-history index cards; Fergus's old-settler death notices, and every one of those readings is a committed refusal on the forename or the initial.</t>
+          <t>Reached only by surname in the Newberry index; the old-settler notices — every one a committed refusal on the forename.</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -1863,14 +1847,10 @@
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
-          <t>'Alison B. Vaughn' and 'Alanson B. Vaughan' are the same initial and middle initial under two spellings of one surname, in the same list family; the 1830 schedule's 'James Vaughn' is refused on the forename.</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>No independent record carries either spelling in Chicago, so the pair stays two rows rather than becoming one man.</t>
-        </is>
-      </c>
+          <t>A same-name lead, unasserted: cand_vaughan_vaughn_same_hand.</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
           <t>chicago_democrat_1833_1835</t>
@@ -1889,7 +1869,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>research-only; candidate retained unasserted; no grade, household or placement is moved by this row</t>
+          <t>candidate retained unasserted; no grade or placement moves</t>
         </is>
       </c>
     </row>
@@ -1923,7 +1903,7 @@
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the 1830 Peoria/Putnam schedule leaves for the Chicago precinct; the 1840 census heads read for this project; the St Mary's and St Cyr registers; the 1833-1835 Chicago poll, tax and voter rolls (IRAD); Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the transcribed county-history corpus; the Newberry family-history index cards; Fergus's old-settler death notices.</t>
+          <t>Named independently of the post-office lists in the 1830 schedule; the 1840 census; the parish registers; the civic rolls; the directories; the county histories; the Newberry index; the old-settler notices.</t>
         </is>
       </c>
       <c r="I26" t="inlineStr"/>
@@ -1949,7 +1929,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -1987,14 +1967,10 @@
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Fergus 1839 prints 'Avery, Charles E., lumber dealer, cor. LaSalle and So. Water'.</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>The directory's man carries a middle initial the letter list does not, and the 1840 reading's 'C. E. Avery' is refused against 'Charles Avery' on the forename in the committed crosswalk.</t>
-        </is>
-      </c>
+          <t>A same-name lead, unasserted: cand_charles_e_avery_lumber.</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
           <t>fergus_chicago_directory_1839</t>
@@ -2017,7 +1993,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>research-only; candidate retained unasserted; no grade, household or placement is moved by this row</t>
+          <t>candidate retained unasserted; no grade or placement moves</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2028,7 @@
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Reached only by surname in the Newberry family-history index cards, and every one of those readings is a committed refusal on the forename or the initial.</t>
+          <t>Reached only by surname in the Newberry index — every one a committed refusal on the forename.</t>
         </is>
       </c>
       <c r="J28" t="inlineStr"/>
@@ -2103,7 +2079,7 @@
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the 1830 Peoria/Putnam schedule leaves for the Chicago precinct; the 1840 census heads read for this project; the St Mary's and St Cyr registers; the 1833-1835 Chicago poll, tax and voter rolls (IRAD); Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the transcribed county-history corpus; the Illinois public-domain land tract sales entries held here; the Newberry family-history index cards; Fergus's old-settler death notices.</t>
+          <t>Named independently of the post-office lists in the 1830 schedule; the 1840 census; the parish registers; the civic rolls; the directories; the county histories; the land sales; the Newberry index; the old-settler notices.</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
@@ -2129,7 +2105,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -2164,7 +2140,7 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Reached only by surname in Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; Fergus's old-settler death notices, and every one of those readings is a committed refusal on the forename or the initial.</t>
+          <t>Reached only by surname in the directories; the old-settler notices — every one a committed refusal on the forename.</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
@@ -2216,7 +2192,7 @@
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Not reached at all outside the post-office lists: no committed corpus carries the name.</t>
+          <t>Not reached outside the post-office lists.</t>
         </is>
       </c>
       <c r="J31" t="inlineStr"/>
@@ -2267,7 +2243,7 @@
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the 1830 Peoria/Putnam schedule leaves for the Chicago precinct; the 1840 census heads read for this project; the St Mary's and St Cyr registers; the 1833-1835 Chicago poll, tax and voter rolls (IRAD); Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the transcribed county-history corpus; the Illinois public-domain land tract sales entries held here; the Newberry family-history index cards; Fergus's old-settler death notices.</t>
+          <t>Named independently of the post-office lists in the 1830 schedule; the 1840 census; the parish registers; the civic rolls; the directories; the county histories; the land sales; the Newberry index; the old-settler notices.</t>
         </is>
       </c>
       <c r="I32" t="inlineStr"/>
@@ -2293,7 +2269,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -2331,14 +2307,10 @@
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Joseph Bailly the American Fur Company trader is licensed for the Lake Michigan trade in 1821 (Hurlbut) and Fergus's old-settler death notices print 'Bailly, Joseph, died, Baillytown, Ind., December 21, 1835, aged 61'.</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>Bailly's household stood on the Little Calumet in Indiana, not in Chicago; a letter waiting at the Chicago post office is consistent with a trader who collected mail there and is not evidence of residence.</t>
-        </is>
-      </c>
+          <t>A same-name lead, unasserted: cand_joseph_bailly_baillytown.</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
           <t>nps_bailly_homestead;fergus_historical_series_26_29</t>
@@ -2361,7 +2333,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>research-only; candidate retained unasserted; no grade, household or placement is moved by this row</t>
+          <t>candidate retained unasserted; no grade or placement moves</t>
         </is>
       </c>
     </row>
@@ -2399,14 +2371,10 @@
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
-          <t>'Alonzo Murray' and 'Alonzo Murry' differ by one letter in the same list family.</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>Committed refusals stand against every other Murray reached: 'John Murray' in the St Mary's register, 'Patrick Murray' on the 1834 poll, 'Alon On Sweet' in Fergus 1839 — each a surname-only or forename-conflict refusal.</t>
-        </is>
-      </c>
+          <t>A same-name lead, unasserted: cand_murray_murry_same_hand.</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
           <t>chicago_democrat_1833_1835</t>
@@ -2425,7 +2393,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>research-only; candidate retained unasserted; no grade, household or placement is moved by this row</t>
+          <t>candidate retained unasserted; no grade or placement moves</t>
         </is>
       </c>
     </row>
@@ -2459,7 +2427,7 @@
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the committed source records cited.</t>
+          <t>Named independently of the post-office lists in the sources cited.</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
@@ -2485,7 +2453,7 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -2520,7 +2488,7 @@
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Not reached at all outside the post-office lists: no committed corpus carries the name.</t>
+          <t>Not reached outside the post-office lists.</t>
         </is>
       </c>
       <c r="J36" t="inlineStr"/>
@@ -2575,14 +2543,10 @@
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
-          <t>'Alonzo Murry' and 'Alonzo Murray' differ by one letter in the same list family; the St Cyr register's 1837 'S. Murry' is refused on the forename.</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>The Murray surname is common in this corpus (James H, Patrick, John are all separately held) and no source equates the two Alonzos.</t>
-        </is>
-      </c>
+          <t>A same-name lead, unasserted: cand_murray_murry_same_hand.</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
           <t>chicago_democrat_1833_1835</t>
@@ -2601,7 +2565,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>research-only; candidate retained unasserted; no grade, household or placement is moved by this row</t>
+          <t>candidate retained unasserted; no grade or placement moves</t>
         </is>
       </c>
     </row>
@@ -2635,7 +2599,7 @@
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the digitised books corpus (Andreas, Hurlbut, Fergus's Historical Series, Hubbard); the 1840 census heads read for this project; the 1833-1835 Chicago poll, tax and voter rolls (IRAD); Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the transcribed county-history corpus; the Newberry family-history index cards.</t>
+          <t>Named independently of the post-office lists in the books corpus; the 1840 census; the civic rolls; the directories; the county histories; the Newberry index.</t>
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
@@ -2661,7 +2625,7 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -2696,7 +2660,7 @@
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Not reached at all outside the post-office lists: no committed corpus carries the name.</t>
+          <t>Not reached outside the post-office lists.</t>
         </is>
       </c>
       <c r="J39" t="inlineStr"/>
@@ -2748,7 +2712,7 @@
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Reached only by surname in the Newberry family-history index cards, and every one of those readings is a committed refusal on the forename or the initial.</t>
+          <t>Reached only by surname in the Newberry index — every one a committed refusal on the forename.</t>
         </is>
       </c>
       <c r="J40" t="inlineStr"/>
@@ -2799,7 +2763,7 @@
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the digitised books corpus (Andreas, Hurlbut, Fergus's Historical Series, Hubbard); the 1840 census heads read for this project; the 1833-1835 Chicago poll, tax and voter rolls (IRAD); Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the transcribed county-history corpus; the Illinois public-domain land tract sales entries held here; the Newberry family-history index cards; Fergus's old-settler death notices.</t>
+          <t>Named independently of the post-office lists in the books corpus; the 1840 census; the civic rolls; the directories; the county histories; the land sales; the Newberry index; the old-settler notices.</t>
         </is>
       </c>
       <c r="I41" t="inlineStr"/>
@@ -2825,7 +2789,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -2860,7 +2824,7 @@
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Not reached at all outside the post-office lists: no committed corpus carries the name.</t>
+          <t>Not reached outside the post-office lists.</t>
         </is>
       </c>
       <c r="J42" t="inlineStr"/>
@@ -2915,14 +2879,10 @@
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
-          <t>A community history dates Alva Dunlap's first Illinois journey to 1834 and his settlement near Peoria.</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>Peoria is not Chicago and the account names no Chicago residence; the surname stands in Fergus 1839, Fergus 1843 and Norris 1844 with no entry carrying the initial A.</t>
-        </is>
-      </c>
+          <t>A same-name lead, unasserted: cand_alva_dunlap_peoria.</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
           <t>dunlap_alva_dunlap_history</t>
@@ -2945,7 +2905,7 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>research-only; candidate retained unasserted; no grade, household or placement is moved by this row</t>
+          <t>candidate retained unasserted; no grade or placement moves</t>
         </is>
       </c>
     </row>
@@ -2979,7 +2939,7 @@
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the 1833-1835 Chicago poll, tax and voter rolls (IRAD); Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the transcribed county-history corpus; the Illinois public-domain land tract sales entries held here; the Newberry family-history index cards; Fergus's old-settler death notices.</t>
+          <t>Named independently of the post-office lists in the civic rolls; the directories; the county histories; the land sales; the Newberry index; the old-settler notices.</t>
         </is>
       </c>
       <c r="I44" t="inlineStr"/>
@@ -3005,7 +2965,7 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -3040,7 +3000,7 @@
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Not reached at all outside the post-office lists: no committed corpus carries the name.</t>
+          <t>Not reached outside the post-office lists.</t>
         </is>
       </c>
       <c r="J45" t="inlineStr"/>
@@ -3095,14 +3055,10 @@
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Kaneville Township's history names Amos and Amanda Miner among its settlers.</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>Kane County, and no record ties the pair to the Chicago post office; the Newberry card the sweep reaches is a 'Milner' heading, not 'Miner'.</t>
-        </is>
-      </c>
+          <t>A same-name lead, unasserted: cand_amanda_miner_kaneville.</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr">
         <is>
           <t>kaneville_amanda_miner</t>
@@ -3125,7 +3081,7 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>research-only; candidate retained unasserted; no grade, household or placement is moved by this row</t>
+          <t>candidate retained unasserted; no grade or placement moves</t>
         </is>
       </c>
     </row>
@@ -3159,7 +3115,7 @@
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the digitised books corpus (Andreas, Hurlbut, Fergus's Historical Series, Hubbard); the 1833-1835 Chicago poll, tax and voter rolls (IRAD); Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the transcribed county-history corpus; the Illinois public-domain land tract sales entries held here; Fergus's old-settler death notices.</t>
+          <t>Named independently of the post-office lists in the books corpus; the civic rolls; the directories; the county histories; the land sales; the old-settler notices.</t>
         </is>
       </c>
       <c r="I47" t="inlineStr"/>
@@ -3185,7 +3141,7 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -3220,7 +3176,7 @@
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Reached only by surname in the Newberry family-history index cards, and every one of those readings is a committed refusal on the forename or the initial.</t>
+          <t>Reached only by surname in the Newberry index — every one a committed refusal on the forename.</t>
         </is>
       </c>
       <c r="J48" t="inlineStr"/>
@@ -3272,7 +3228,7 @@
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Reached only by surname in the Newberry family-history index cards, and every one of those readings is a committed refusal on the forename or the initial.</t>
+          <t>Reached only by surname in the Newberry index — every one a committed refusal on the forename.</t>
         </is>
       </c>
       <c r="J49" t="inlineStr"/>
@@ -3323,7 +3279,7 @@
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the digitised books corpus (Andreas, Hurlbut, Fergus's Historical Series, Hubbard); the 1833-1835 Chicago poll, tax and voter rolls (IRAD); Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the transcribed county-history corpus; the Newberry family-history index cards; Fergus's old-settler death notices.</t>
+          <t>Named independently of the post-office lists in the books corpus; the civic rolls; the directories; the county histories; the Newberry index; the old-settler notices.</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
@@ -3349,7 +3305,7 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -3384,7 +3340,7 @@
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Not reached at all outside the post-office lists: no committed corpus carries the name.</t>
+          <t>Not reached outside the post-office lists.</t>
         </is>
       </c>
       <c r="J51" t="inlineStr"/>
@@ -3436,7 +3392,7 @@
       <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Reached only by surname in the Illinois public-domain land tract sales entries held here, and every one of those readings is a committed refusal on the forename or the initial.</t>
+          <t>Reached only by surname in the land sales — every one a committed refusal on the forename.</t>
         </is>
       </c>
       <c r="J52" t="inlineStr"/>
@@ -3487,7 +3443,7 @@
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the digitised books corpus (Andreas, Hurlbut, Fergus's Historical Series, Hubbard); the 1840 census heads read for this project; the 1833-1835 Chicago poll, tax and voter rolls (IRAD); Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the transcribed county-history corpus; the Illinois public-domain land tract sales entries held here; the Newberry family-history index cards.</t>
+          <t>Named independently of the post-office lists in the books corpus; the 1840 census; the civic rolls; the directories; the county histories; the land sales; the Newberry index.</t>
         </is>
       </c>
       <c r="I53" t="inlineStr"/>
@@ -3513,7 +3469,7 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -3548,7 +3504,7 @@
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Reached only by surname in Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the Illinois public-domain land tract sales entries held here; the Newberry family-history index cards, and every one of those readings is a committed refusal on the forename or the initial.</t>
+          <t>Reached only by surname in the directories; the land sales; the Newberry index — every one a committed refusal on the forename.</t>
         </is>
       </c>
       <c r="J54" t="inlineStr"/>
@@ -3603,14 +3559,10 @@
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
-          <t>A Kane County township history recalls an Andrew Miles (or Mills) claim of 1834.</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>The same passage carries a Miles/Mills spelling conflict, and Fergus 1843 and Norris 1844 both refuse the surname on the initial.</t>
-        </is>
-      </c>
+          <t>A same-name lead, unasserted: cand_andrew_miles_geneva.</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
           <t>kane_geneva_andrew_miles</t>
@@ -3633,7 +3585,7 @@
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>research-only; candidate retained unasserted; no grade, household or placement is moved by this row</t>
+          <t>candidate retained unasserted; no grade or placement moves</t>
         </is>
       </c>
     </row>
@@ -3667,7 +3619,7 @@
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the 1830 Peoria/Putnam schedule leaves for the Chicago precinct; the 1833-1835 Chicago poll, tax and voter rolls (IRAD); the transcribed county-history corpus; the Illinois public-domain land tract sales entries held here.</t>
+          <t>Named independently of the post-office lists in the 1830 schedule; the civic rolls; the county histories; the land sales.</t>
         </is>
       </c>
       <c r="I56" t="inlineStr"/>
@@ -3693,7 +3645,7 @@
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -3728,7 +3680,7 @@
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Not reached at all outside the post-office lists: no committed corpus carries the name.</t>
+          <t>Not reached outside the post-office lists.</t>
         </is>
       </c>
       <c r="J57" t="inlineStr"/>
@@ -3780,7 +3732,7 @@
       <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Not reached at all outside the post-office lists: no committed corpus carries the name.</t>
+          <t>Not reached outside the post-office lists.</t>
         </is>
       </c>
       <c r="J58" t="inlineStr"/>
@@ -3831,7 +3783,7 @@
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the digitised books corpus (Andreas, Hurlbut, Fergus's Historical Series, Hubbard); Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the transcribed county-history corpus; the Newberry family-history index cards; Fergus's old-settler death notices.</t>
+          <t>Named independently of the post-office lists in the books corpus; the directories; the county histories; the Newberry index; the old-settler notices.</t>
         </is>
       </c>
       <c r="I59" t="inlineStr"/>
@@ -3857,7 +3809,7 @@
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -3895,14 +3847,10 @@
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Fergus 1839 carries a Bishop on Illinois street whose surname folds to this one and whose given name agrees on the initial J.</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>Illinois Street is a Kinzie's Addition name the 1835 street layer does not carry, so the entry cannot even be placed in the modelled town, and the 1837 poll refuses the surname on the initial.</t>
-        </is>
-      </c>
+          <t>A same-name lead, unasserted: cand_j_e_bishop_1839_illinois_st.</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr"/>
       <c r="J60" t="inlineStr">
         <is>
           <t>fergus_chicago_directory_1839</t>
@@ -3925,7 +3873,7 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>research-only; candidate retained unasserted; no grade, household or placement is moved by this row</t>
+          <t>candidate retained unasserted; no grade or placement moves</t>
         </is>
       </c>
     </row>
@@ -3960,7 +3908,7 @@
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Reached only by surname in the Newberry family-history index cards, and every one of those readings is a committed refusal on the forename or the initial.</t>
+          <t>Reached only by surname in the Newberry index — every one a committed refusal on the forename.</t>
         </is>
       </c>
       <c r="J61" t="inlineStr"/>
@@ -4011,7 +3959,7 @@
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the digitised books corpus (Andreas, Hurlbut, Fergus's Historical Series, Hubbard); the 1833-1835 Chicago poll, tax and voter rolls (IRAD); Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the transcribed county-history corpus.</t>
+          <t>Named independently of the post-office lists in the books corpus; the civic rolls; the directories; the county histories.</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
@@ -4037,7 +3985,7 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -4075,14 +4023,10 @@
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
-          <t>A William G. Blair stands among the first settlers rostered for Winnebago County in 1835-36.</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>Fergus 1843's Chicago hardware Blair is 'Blair, William' of 111 S. Water with no middle initial and a documented later arrival; the Winnebago roster is a different county and neither bridges the 1834-35 Chicago postal entry.</t>
-        </is>
-      </c>
+          <t>A same-name lead, unasserted: cand_william_g_blair_winnebago.</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr">
         <is>
           <t>rockford_first_settlers_1835</t>
@@ -4105,7 +4049,7 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>research-only; candidate retained unasserted; no grade, household or placement is moved by this row</t>
+          <t>candidate retained unasserted; no grade or placement moves</t>
         </is>
       </c>
     </row>
@@ -4140,7 +4084,7 @@
       <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Not reached at all outside the post-office lists: no committed corpus carries the name.</t>
+          <t>Not reached outside the post-office lists.</t>
         </is>
       </c>
       <c r="J64" t="inlineStr"/>
@@ -4191,7 +4135,7 @@
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the digitised books corpus (Andreas, Hurlbut, Fergus's Historical Series, Hubbard); the 1840 census heads read for this project; Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the transcribed county-history corpus; the Newberry family-history index cards.</t>
+          <t>Named independently of the post-office lists in the books corpus; the 1840 census; the directories; the county histories; the Newberry index.</t>
         </is>
       </c>
       <c r="I65" t="inlineStr"/>
@@ -4217,7 +4161,7 @@
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4196,7 @@
       <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr">
         <is>
-          <t>Reached only by surname in the Newberry family-history index cards, and every one of those readings is a committed refusal on the forename or the initial.</t>
+          <t>Reached only by surname in the Newberry index — every one a committed refusal on the forename.</t>
         </is>
       </c>
       <c r="J66" t="inlineStr"/>
@@ -4304,7 +4248,7 @@
       <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
-          <t>Reached only by surname in the 1840 census heads read for this project; Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the Newberry family-history index cards; Fergus's old-settler death notices, and every one of those readings is a committed refusal on the forename or the initial.</t>
+          <t>Reached only by surname in the 1840 census; the directories; the Newberry index; the old-settler notices — every one a committed refusal on the forename.</t>
         </is>
       </c>
       <c r="J67" t="inlineStr"/>
@@ -4355,7 +4299,7 @@
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the transcribed county-history corpus; the Newberry family-history index cards; Fergus's old-settler death notices.</t>
+          <t>Named independently of the post-office lists in the directories; the county histories; the Newberry index; the old-settler notices.</t>
         </is>
       </c>
       <c r="I68" t="inlineStr"/>
@@ -4381,7 +4325,7 @@
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -4416,7 +4360,7 @@
       <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Reached only by surname in the Newberry family-history index cards, and every one of those readings is a committed refusal on the forename or the initial.</t>
+          <t>Reached only by surname in the Newberry index — every one a committed refusal on the forename.</t>
         </is>
       </c>
       <c r="J69" t="inlineStr"/>
@@ -4471,14 +4415,10 @@
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
-          <t>'Aron Parcell' and 'Aaron Parcel' are two post-office readings one letter apart, in the same list family.</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>Nothing outside the letter lists names either spelling; collapsing them would assert an identity no source states.</t>
-        </is>
-      </c>
+          <t>A same-name lead, unasserted: cand_parcel_parcell_same_hand.</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr"/>
       <c r="J70" t="inlineStr">
         <is>
           <t>chicago_democrat_1833_1835</t>
@@ -4497,7 +4437,7 @@
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>research-only; candidate retained unasserted; no grade, household or placement is moved by this row</t>
+          <t>candidate retained unasserted; no grade or placement moves</t>
         </is>
       </c>
     </row>
@@ -4531,7 +4471,7 @@
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the digitised books corpus (Andreas, Hurlbut, Fergus's Historical Series, Hubbard); the 1840 census heads read for this project; the 1833-1835 Chicago poll, tax and voter rolls (IRAD); Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the transcribed county-history corpus; the Illinois public-domain land tract sales entries held here; the Newberry family-history index cards.</t>
+          <t>Named independently of the post-office lists in the books corpus; the 1840 census; the civic rolls; the directories; the county histories; the land sales; the Newberry index.</t>
         </is>
       </c>
       <c r="I71" t="inlineStr"/>
@@ -4557,7 +4497,7 @@
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -4595,14 +4535,10 @@
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
-          <t>The Firelands Pioneer of 1888 carries an exact-name Rouse Bly in Huron County, Ohio.</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>A competing Ohio identity of the same uncommon name is a reason for caution, not a bridge; nothing in the Chicago corpus repeats the name.</t>
-        </is>
-      </c>
+          <t>A same-name lead, unasserted: cand_rouse_bly_firelands.</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr"/>
       <c r="J72" t="inlineStr">
         <is>
           <t>ohio_firelands_rouse_bly</t>
@@ -4625,7 +4561,7 @@
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>research-only; candidate retained unasserted; no grade, household or placement is moved by this row</t>
+          <t>candidate retained unasserted; no grade or placement moves</t>
         </is>
       </c>
     </row>
@@ -4660,7 +4596,7 @@
       <c r="H73" t="inlineStr"/>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Not reached at all outside the post-office lists: no committed corpus carries the name.</t>
+          <t>Not reached outside the post-office lists.</t>
         </is>
       </c>
       <c r="J73" t="inlineStr"/>
@@ -4711,7 +4647,7 @@
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the 1840 census heads read for this project; the 1833-1835 Chicago poll, tax and voter rolls (IRAD); Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the Newberry family-history index cards.</t>
+          <t>Named independently of the post-office lists in the 1840 census; the civic rolls; the directories; the Newberry index.</t>
         </is>
       </c>
       <c r="I74" t="inlineStr"/>
@@ -4737,7 +4673,7 @@
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>
@@ -4772,7 +4708,7 @@
       <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Reached only by surname in the 1840 census heads read for this project; Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844, and every one of those readings is a committed refusal on the forename or the initial.</t>
+          <t>Reached only by surname in the 1840 census; the directories — every one a committed refusal on the forename.</t>
         </is>
       </c>
       <c r="J75" t="inlineStr"/>
@@ -4824,7 +4760,7 @@
       <c r="H76" t="inlineStr"/>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Not reached at all outside the post-office lists: no committed corpus carries the name.</t>
+          <t>Not reached outside the post-office lists.</t>
         </is>
       </c>
       <c r="J76" t="inlineStr"/>
@@ -4875,7 +4811,7 @@
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Named independently of the post-office lists in the digitised books corpus (Andreas, Hurlbut, Fergus's Historical Series, Hubbard); the 1833-1835 Chicago poll, tax and voter rolls (IRAD); Fergus's Chicago directories of 1839 and 1843 and Norris's of 1844; the transcribed county-history corpus; the Illinois public-domain land tract sales entries held here; the Newberry family-history index cards.</t>
+          <t>Named independently of the post-office lists in the books corpus; the civic rolls; the directories; the county histories; the land sales; the Newberry index.</t>
         </is>
       </c>
       <c r="I77" t="inlineStr"/>
@@ -4901,7 +4837,7 @@
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>Established profile; the row records the corroboration this person already stood on and asserts no new fact.</t>
+          <t>records corroboration already standing; asserts no new fact</t>
         </is>
       </c>
     </row>

</xml_diff>